<commit_message>
#2 U4 update in BOM
</commit_message>
<xml_diff>
--- a/Design-Files/BOM/eSpark BOM.xlsx
+++ b/Design-Files/BOM/eSpark BOM.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="320">
   <si>
     <t>Component list</t>
   </si>
@@ -928,7 +928,10 @@
     <t>SOP-8</t>
   </si>
   <si>
-    <t>AT24C16D-SSHM-B</t>
+    <t>FT24C16A-ESR-T</t>
+  </si>
+  <si>
+    <t>FMD</t>
   </si>
   <si>
     <t>C615460</t>
@@ -2783,7 +2786,7 @@
       <c r="R8" s="28"/>
       <c r="S8" s="64"/>
     </row>
-    <row r="9" spans="1:19">
+    <row r="9" ht="15.15" spans="1:19">
       <c r="A9" s="2"/>
       <c r="B9" s="33" t="s">
         <v>7</v>
@@ -2843,7 +2846,7 @@
     <row r="10" ht="24" spans="1:19">
       <c r="A10" s="2"/>
       <c r="B10" s="34">
-        <f>ROW(B10)-ROW($B$9)</f>
+        <f t="shared" ref="B10:B17" si="0">ROW(B10)-ROW($B$9)</f>
         <v>1</v>
       </c>
       <c r="C10" s="35" t="s">
@@ -2877,7 +2880,7 @@
         <v>1</v>
       </c>
       <c r="M10" s="36">
-        <f>L10*5</f>
+        <f t="shared" ref="M10:M17" si="1">L10*5</f>
         <v>5</v>
       </c>
       <c r="N10" s="36">
@@ -2890,7 +2893,7 @@
         <v>0.0347</v>
       </c>
       <c r="Q10" s="55">
-        <f>P10*N10</f>
+        <f t="shared" ref="Q10:Q17" si="2">P10*N10</f>
         <v>0.347</v>
       </c>
       <c r="R10" s="36"/>
@@ -2899,7 +2902,7 @@
     <row r="11" spans="1:19">
       <c r="A11" s="2"/>
       <c r="B11" s="37">
-        <f>ROW(B11)-ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="C11" s="38" t="s">
@@ -2933,7 +2936,7 @@
         <v>5</v>
       </c>
       <c r="M11" s="39">
-        <f>L11*5</f>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="N11" s="39">
@@ -2946,7 +2949,7 @@
         <v>0.0034</v>
       </c>
       <c r="Q11" s="57">
-        <f>P11*N11</f>
+        <f t="shared" si="2"/>
         <v>0.34</v>
       </c>
       <c r="R11" s="39"/>
@@ -2955,7 +2958,7 @@
     <row r="12" ht="36" spans="1:19">
       <c r="A12" s="2"/>
       <c r="B12" s="34">
-        <f>ROW(B12)-ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C12" s="35" t="s">
@@ -2989,7 +2992,7 @@
         <v>1</v>
       </c>
       <c r="M12" s="36">
-        <f>L12*5</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="N12" s="36">
@@ -3002,7 +3005,7 @@
         <v>0.0716</v>
       </c>
       <c r="Q12" s="55">
-        <f>P12*N12</f>
+        <f t="shared" si="2"/>
         <v>0.716</v>
       </c>
       <c r="R12" s="36"/>
@@ -3011,7 +3014,7 @@
     <row r="13" spans="1:19">
       <c r="A13" s="2"/>
       <c r="B13" s="37">
-        <f>ROW(B13)-ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C13" s="35" t="s">
@@ -3045,7 +3048,7 @@
         <v>3</v>
       </c>
       <c r="M13" s="39">
-        <f>L13*5</f>
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
       <c r="N13" s="39">
@@ -3058,7 +3061,7 @@
         <v>0.0239</v>
       </c>
       <c r="Q13" s="57">
-        <f>P13*N13</f>
+        <f t="shared" si="2"/>
         <v>0.478</v>
       </c>
       <c r="R13" s="39"/>
@@ -3067,7 +3070,7 @@
     <row r="14" ht="24" spans="1:19">
       <c r="A14" s="2"/>
       <c r="B14" s="34">
-        <f>ROW(B14)-ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C14" s="35" t="s">
@@ -3101,7 +3104,7 @@
         <v>1</v>
       </c>
       <c r="M14" s="36">
-        <f>L14*5</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="N14" s="36">
@@ -3114,7 +3117,7 @@
         <v>0.0027</v>
       </c>
       <c r="Q14" s="55">
-        <f>P14*N14</f>
+        <f t="shared" si="2"/>
         <v>0.27</v>
       </c>
       <c r="R14" s="36"/>
@@ -3123,7 +3126,7 @@
     <row r="15" ht="36" spans="1:19">
       <c r="A15" s="2"/>
       <c r="B15" s="37">
-        <f>ROW(B15)-ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C15" s="38" t="s">
@@ -3157,7 +3160,7 @@
         <v>1</v>
       </c>
       <c r="M15" s="39">
-        <f>L15*5</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="N15" s="39">
@@ -3170,7 +3173,7 @@
         <v>0.0236</v>
       </c>
       <c r="Q15" s="57">
-        <f>P15*N15</f>
+        <f t="shared" si="2"/>
         <v>0.472</v>
       </c>
       <c r="R15" s="39"/>
@@ -3179,7 +3182,7 @@
     <row r="16" spans="1:19">
       <c r="A16" s="2"/>
       <c r="B16" s="34">
-        <f>ROW(B16)-ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C16" s="35" t="s">
@@ -3213,7 +3216,7 @@
         <v>6</v>
       </c>
       <c r="M16" s="36">
-        <f>L16*5</f>
+        <f t="shared" si="1"/>
         <v>30</v>
       </c>
       <c r="N16" s="36">
@@ -3226,7 +3229,7 @@
         <v>0.0886</v>
       </c>
       <c r="Q16" s="55">
-        <f>P16*N16</f>
+        <f t="shared" si="2"/>
         <v>3.101</v>
       </c>
       <c r="R16" s="36"/>
@@ -3235,7 +3238,7 @@
     <row r="17" ht="24" spans="1:19">
       <c r="A17" s="2"/>
       <c r="B17" s="37">
-        <f>ROW(B17)-ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C17" s="38" t="s">
@@ -3269,7 +3272,7 @@
         <v>1</v>
       </c>
       <c r="M17" s="39">
-        <f>L17*5</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="N17" s="39">
@@ -3282,7 +3285,7 @@
         <v>0.0304</v>
       </c>
       <c r="Q17" s="57">
-        <f>P17*N17</f>
+        <f t="shared" si="2"/>
         <v>0.608</v>
       </c>
       <c r="R17" s="39"/>
@@ -3291,7 +3294,7 @@
     <row r="18" ht="24" spans="1:19">
       <c r="A18" s="2"/>
       <c r="B18" s="37">
-        <f t="shared" ref="B18:B59" si="0">ROW(B18)-ROW($B$9)</f>
+        <f t="shared" ref="B18:B59" si="3">ROW(B18)-ROW($B$9)</f>
         <v>9</v>
       </c>
       <c r="C18" s="38" t="s">
@@ -3325,7 +3328,7 @@
         <v>3</v>
       </c>
       <c r="M18" s="39">
-        <f t="shared" ref="M18:M59" si="1">L18*5</f>
+        <f t="shared" ref="M18:M59" si="4">L18*5</f>
         <v>15</v>
       </c>
       <c r="N18" s="39">
@@ -3338,7 +3341,7 @@
         <v>0.0088</v>
       </c>
       <c r="Q18" s="57">
-        <f t="shared" ref="Q18:Q59" si="2">P18*N18</f>
+        <f t="shared" ref="Q18:Q59" si="5">P18*N18</f>
         <v>0.44</v>
       </c>
       <c r="R18" s="39"/>
@@ -3347,7 +3350,7 @@
     <row r="19" spans="1:19">
       <c r="A19" s="2"/>
       <c r="B19" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>10</v>
       </c>
       <c r="C19" s="38" t="s">
@@ -3381,7 +3384,7 @@
         <v>1</v>
       </c>
       <c r="M19" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N19" s="36">
@@ -3394,7 +3397,7 @@
         <v>0.1784</v>
       </c>
       <c r="Q19" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>1.784</v>
       </c>
       <c r="R19" s="36"/>
@@ -3403,7 +3406,7 @@
     <row r="20" ht="36" spans="1:19">
       <c r="A20" s="2"/>
       <c r="B20" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>11</v>
       </c>
       <c r="C20" s="38" t="s">
@@ -3437,7 +3440,7 @@
         <v>18</v>
       </c>
       <c r="M20" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>90</v>
       </c>
       <c r="N20" s="39">
@@ -3450,7 +3453,7 @@
         <v>0.0121</v>
       </c>
       <c r="Q20" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>1.21</v>
       </c>
       <c r="R20" s="39"/>
@@ -3459,7 +3462,7 @@
     <row r="21" ht="48" spans="1:19">
       <c r="A21" s="2"/>
       <c r="B21" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>12</v>
       </c>
       <c r="C21" s="35" t="s">
@@ -3491,7 +3494,7 @@
         <v>1</v>
       </c>
       <c r="M21" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N21" s="36">
@@ -3504,7 +3507,7 @@
         <v>0.2446</v>
       </c>
       <c r="Q21" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.446</v>
       </c>
       <c r="R21" s="36"/>
@@ -3513,7 +3516,7 @@
     <row r="22" ht="48" spans="1:19">
       <c r="A22" s="2"/>
       <c r="B22" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>13</v>
       </c>
       <c r="C22" s="38" t="s">
@@ -3545,7 +3548,7 @@
         <v>1</v>
       </c>
       <c r="M22" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N22" s="39">
@@ -3558,7 +3561,7 @@
         <v>0.4296</v>
       </c>
       <c r="Q22" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.5776</v>
       </c>
       <c r="R22" s="39"/>
@@ -3567,7 +3570,7 @@
     <row r="23" ht="24" spans="1:19">
       <c r="A23" s="2"/>
       <c r="B23" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>14</v>
       </c>
       <c r="C23" s="35" t="s">
@@ -3599,7 +3602,7 @@
         <v>1</v>
       </c>
       <c r="M23" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N23" s="36">
@@ -3612,7 +3615,7 @@
         <v>0.024</v>
       </c>
       <c r="Q23" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.48</v>
       </c>
       <c r="R23" s="36"/>
@@ -3621,7 +3624,7 @@
     <row r="24" ht="36" spans="1:19">
       <c r="A24" s="2"/>
       <c r="B24" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>15</v>
       </c>
       <c r="C24" s="38" t="s">
@@ -3653,7 +3656,7 @@
         <v>1</v>
       </c>
       <c r="M24" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N24" s="39">
@@ -3666,7 +3669,7 @@
         <v>0.0369</v>
       </c>
       <c r="Q24" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.369</v>
       </c>
       <c r="R24" s="39"/>
@@ -3675,7 +3678,7 @@
     <row r="25" spans="1:19">
       <c r="A25" s="2"/>
       <c r="B25" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>16</v>
       </c>
       <c r="C25" s="35" t="s">
@@ -3707,7 +3710,7 @@
         <v>1</v>
       </c>
       <c r="M25" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N25" s="36">
@@ -3720,7 +3723,7 @@
         <v>0.0493</v>
       </c>
       <c r="Q25" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.493</v>
       </c>
       <c r="R25" s="36"/>
@@ -3729,7 +3732,7 @@
     <row r="26" ht="24" spans="1:19">
       <c r="A26" s="2"/>
       <c r="B26" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
       <c r="C26" s="38" t="s">
@@ -3761,7 +3764,7 @@
         <v>1</v>
       </c>
       <c r="M26" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N26" s="39">
@@ -3774,7 +3777,7 @@
         <v>0.024</v>
       </c>
       <c r="Q26" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.48</v>
       </c>
       <c r="R26" s="39"/>
@@ -3783,7 +3786,7 @@
     <row r="27" ht="36" spans="1:19">
       <c r="A27" s="2"/>
       <c r="B27" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>18</v>
       </c>
       <c r="C27" s="42" t="s">
@@ -3817,7 +3820,7 @@
         <v>1</v>
       </c>
       <c r="M27" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N27" s="41" t="s">
@@ -3840,7 +3843,7 @@
     <row r="28" ht="24" spans="1:19">
       <c r="A28" s="2"/>
       <c r="B28" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>19</v>
       </c>
       <c r="C28" s="38" t="s">
@@ -3874,7 +3877,7 @@
         <v>1</v>
       </c>
       <c r="M28" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N28" s="39">
@@ -3887,7 +3890,7 @@
         <v>0.8035</v>
       </c>
       <c r="Q28" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>4.821</v>
       </c>
       <c r="R28" s="39"/>
@@ -3896,7 +3899,7 @@
     <row r="29" ht="24" spans="1:19">
       <c r="A29" s="2"/>
       <c r="B29" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="C29" s="42" t="s">
@@ -3930,7 +3933,7 @@
         <v>2</v>
       </c>
       <c r="M29" s="41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="N29" s="41" t="s">
@@ -3953,7 +3956,7 @@
     <row r="30" ht="36" spans="1:19">
       <c r="A30" s="2"/>
       <c r="B30" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>21</v>
       </c>
       <c r="C30" s="38" t="s">
@@ -3987,7 +3990,7 @@
         <v>1</v>
       </c>
       <c r="M30" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N30" s="39">
@@ -4000,7 +4003,7 @@
         <v>0.1704</v>
       </c>
       <c r="Q30" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>1.704</v>
       </c>
       <c r="R30" s="39"/>
@@ -4009,7 +4012,7 @@
     <row r="31" ht="36" spans="1:19">
       <c r="A31" s="2"/>
       <c r="B31" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>22</v>
       </c>
       <c r="C31" s="35" t="s">
@@ -4030,7 +4033,9 @@
       <c r="H31" s="36" t="s">
         <v>150</v>
       </c>
-      <c r="I31" s="36"/>
+      <c r="I31" s="36" t="s">
+        <v>31</v>
+      </c>
       <c r="J31" s="36" t="s">
         <v>151</v>
       </c>
@@ -4041,7 +4046,7 @@
         <v>1</v>
       </c>
       <c r="M31" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N31" s="36">
@@ -4054,7 +4059,7 @@
         <v>0.0317</v>
       </c>
       <c r="Q31" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.634</v>
       </c>
       <c r="R31" s="36"/>
@@ -4063,7 +4068,7 @@
     <row r="32" spans="1:19">
       <c r="A32" s="2"/>
       <c r="B32" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>23</v>
       </c>
       <c r="C32" s="38" t="s">
@@ -4084,7 +4089,9 @@
       <c r="H32" s="39" t="s">
         <v>156</v>
       </c>
-      <c r="I32" s="39"/>
+      <c r="I32" s="36" t="s">
+        <v>31</v>
+      </c>
       <c r="J32" s="39" t="s">
         <v>157</v>
       </c>
@@ -4095,7 +4102,7 @@
         <v>3</v>
       </c>
       <c r="M32" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>15</v>
       </c>
       <c r="N32" s="39">
@@ -4108,7 +4115,7 @@
         <v>1.3714</v>
       </c>
       <c r="Q32" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>21.9424</v>
       </c>
       <c r="R32" s="39"/>
@@ -4117,7 +4124,7 @@
     <row r="33" ht="24" spans="1:19">
       <c r="A33" s="2"/>
       <c r="B33" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>24</v>
       </c>
       <c r="C33" s="35" t="s">
@@ -4138,7 +4145,9 @@
       <c r="H33" s="36" t="s">
         <v>163</v>
       </c>
-      <c r="I33" s="36"/>
+      <c r="I33" s="36" t="s">
+        <v>31</v>
+      </c>
       <c r="J33" s="36" t="s">
         <v>164</v>
       </c>
@@ -4149,7 +4158,7 @@
         <v>8</v>
       </c>
       <c r="M33" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>40</v>
       </c>
       <c r="N33" s="36">
@@ -4162,7 +4171,7 @@
         <v>0.0313</v>
       </c>
       <c r="Q33" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>1.878</v>
       </c>
       <c r="R33" s="36"/>
@@ -4171,7 +4180,7 @@
     <row r="34" ht="24" spans="1:19">
       <c r="A34" s="2"/>
       <c r="B34" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>25</v>
       </c>
       <c r="C34" s="38" t="s">
@@ -4205,7 +4214,7 @@
         <v>2</v>
       </c>
       <c r="M34" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="N34" s="39">
@@ -4218,7 +4227,7 @@
         <v>0.6237</v>
       </c>
       <c r="Q34" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>6.8607</v>
       </c>
       <c r="R34" s="39"/>
@@ -4227,7 +4236,7 @@
     <row r="35" ht="24" spans="1:19">
       <c r="A35" s="2"/>
       <c r="B35" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>26</v>
       </c>
       <c r="C35" s="35" t="s">
@@ -4248,16 +4257,20 @@
       <c r="H35" s="36" t="s">
         <v>177</v>
       </c>
-      <c r="I35" s="36"/>
+      <c r="I35" s="36" t="s">
+        <v>31</v>
+      </c>
       <c r="J35" s="36" t="s">
         <v>178</v>
       </c>
-      <c r="K35" s="36"/>
+      <c r="K35" s="36" t="s">
+        <v>31</v>
+      </c>
       <c r="L35" s="36">
         <v>4</v>
       </c>
       <c r="M35" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>20</v>
       </c>
       <c r="N35" s="36">
@@ -4270,7 +4283,7 @@
         <v>0.0143</v>
       </c>
       <c r="Q35" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.715</v>
       </c>
       <c r="R35" s="36"/>
@@ -4279,7 +4292,7 @@
     <row r="36" ht="27.6" spans="1:19">
       <c r="A36" s="2"/>
       <c r="B36" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>27</v>
       </c>
       <c r="C36" s="35" t="s">
@@ -4313,7 +4326,7 @@
         <v>4</v>
       </c>
       <c r="M36" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>20</v>
       </c>
       <c r="N36" s="39">
@@ -4326,7 +4339,7 @@
         <v>0.0295</v>
       </c>
       <c r="Q36" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>1.18</v>
       </c>
       <c r="R36" s="39"/>
@@ -4335,7 +4348,7 @@
     <row r="37" ht="27.6" spans="1:19">
       <c r="A37" s="2"/>
       <c r="B37" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>28</v>
       </c>
       <c r="C37" s="35" t="s">
@@ -4369,7 +4382,7 @@
         <v>2</v>
       </c>
       <c r="M37" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="N37" s="36">
@@ -4382,7 +4395,7 @@
         <v>0.0186</v>
       </c>
       <c r="Q37" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.93</v>
       </c>
       <c r="R37" s="36"/>
@@ -4391,7 +4404,7 @@
     <row r="38" spans="1:19">
       <c r="A38" s="2"/>
       <c r="B38" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>29</v>
       </c>
       <c r="C38" s="35" t="s">
@@ -4412,7 +4425,9 @@
       <c r="H38" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="I38" s="39"/>
+      <c r="I38" s="39" t="s">
+        <v>31</v>
+      </c>
       <c r="J38" s="39" t="s">
         <v>198</v>
       </c>
@@ -4423,7 +4438,7 @@
         <v>3</v>
       </c>
       <c r="M38" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>15</v>
       </c>
       <c r="N38" s="39">
@@ -4436,7 +4451,7 @@
         <v>0.0135</v>
       </c>
       <c r="Q38" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.675</v>
       </c>
       <c r="R38" s="39"/>
@@ -4445,7 +4460,7 @@
     <row r="39" spans="1:19">
       <c r="A39" s="2"/>
       <c r="B39" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>30</v>
       </c>
       <c r="C39" s="35" t="s">
@@ -4466,7 +4481,9 @@
       <c r="H39" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="I39" s="36"/>
+      <c r="I39" s="39" t="s">
+        <v>31</v>
+      </c>
       <c r="J39" s="36" t="s">
         <v>203</v>
       </c>
@@ -4477,7 +4494,7 @@
         <v>6</v>
       </c>
       <c r="M39" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>30</v>
       </c>
       <c r="N39" s="36">
@@ -4490,7 +4507,7 @@
         <v>0.0012</v>
       </c>
       <c r="Q39" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.12</v>
       </c>
       <c r="R39" s="36"/>
@@ -4499,7 +4516,7 @@
     <row r="40" spans="1:19">
       <c r="A40" s="2"/>
       <c r="B40" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>31</v>
       </c>
       <c r="C40" s="38" t="s">
@@ -4520,7 +4537,9 @@
       <c r="H40" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="I40" s="39"/>
+      <c r="I40" s="39" t="s">
+        <v>31</v>
+      </c>
       <c r="J40" s="39" t="s">
         <v>208</v>
       </c>
@@ -4531,7 +4550,7 @@
         <v>4</v>
       </c>
       <c r="M40" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>20</v>
       </c>
       <c r="N40" s="39">
@@ -4544,7 +4563,7 @@
         <v>0.001</v>
       </c>
       <c r="Q40" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.1</v>
       </c>
       <c r="R40" s="39"/>
@@ -4553,7 +4572,7 @@
     <row r="41" spans="1:19">
       <c r="A41" s="2"/>
       <c r="B41" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>32</v>
       </c>
       <c r="C41" s="38" t="s">
@@ -4574,7 +4593,9 @@
       <c r="H41" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="I41" s="36"/>
+      <c r="I41" s="39" t="s">
+        <v>31</v>
+      </c>
       <c r="J41" s="36" t="s">
         <v>213</v>
       </c>
@@ -4585,7 +4606,7 @@
         <v>2</v>
       </c>
       <c r="M41" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="N41" s="36">
@@ -4598,7 +4619,7 @@
         <v>0.0264</v>
       </c>
       <c r="Q41" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.528</v>
       </c>
       <c r="R41" s="36"/>
@@ -4607,7 +4628,7 @@
     <row r="42" spans="1:19">
       <c r="A42" s="2"/>
       <c r="B42" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>33</v>
       </c>
       <c r="C42" s="38" t="s">
@@ -4628,7 +4649,9 @@
       <c r="H42" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="I42" s="39"/>
+      <c r="I42" s="39" t="s">
+        <v>31</v>
+      </c>
       <c r="J42" s="39" t="s">
         <v>218</v>
       </c>
@@ -4639,7 +4662,7 @@
         <v>3</v>
       </c>
       <c r="M42" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>15</v>
       </c>
       <c r="N42" s="39">
@@ -4652,7 +4675,7 @@
         <v>0.0012</v>
       </c>
       <c r="Q42" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.12</v>
       </c>
       <c r="R42" s="39"/>
@@ -4661,7 +4684,7 @@
     <row r="43" spans="1:19">
       <c r="A43" s="2"/>
       <c r="B43" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>34</v>
       </c>
       <c r="C43" s="35" t="s">
@@ -4682,7 +4705,9 @@
       <c r="H43" s="36" t="s">
         <v>223</v>
       </c>
-      <c r="I43" s="36"/>
+      <c r="I43" s="39" t="s">
+        <v>31</v>
+      </c>
       <c r="J43" s="36" t="s">
         <v>224</v>
       </c>
@@ -4693,7 +4718,7 @@
         <v>6</v>
       </c>
       <c r="M43" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>30</v>
       </c>
       <c r="N43" s="36">
@@ -4706,7 +4731,7 @@
         <v>0.0013</v>
       </c>
       <c r="Q43" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.13</v>
       </c>
       <c r="R43" s="36"/>
@@ -4715,7 +4740,7 @@
     <row r="44" spans="1:19">
       <c r="A44" s="2"/>
       <c r="B44" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>35</v>
       </c>
       <c r="C44" s="38" t="s">
@@ -4736,7 +4761,9 @@
       <c r="H44" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="I44" s="39"/>
+      <c r="I44" s="39" t="s">
+        <v>31</v>
+      </c>
       <c r="J44" s="39" t="s">
         <v>229</v>
       </c>
@@ -4747,7 +4774,7 @@
         <v>2</v>
       </c>
       <c r="M44" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="N44" s="39">
@@ -4760,7 +4787,7 @@
         <v>0.0011</v>
       </c>
       <c r="Q44" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.11</v>
       </c>
       <c r="R44" s="39"/>
@@ -4769,7 +4796,7 @@
     <row r="45" spans="1:19">
       <c r="A45" s="2"/>
       <c r="B45" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>36</v>
       </c>
       <c r="C45" s="35" t="s">
@@ -4790,7 +4817,9 @@
       <c r="H45" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="I45" s="36"/>
+      <c r="I45" s="39" t="s">
+        <v>31</v>
+      </c>
       <c r="J45" s="36" t="s">
         <v>234</v>
       </c>
@@ -4801,7 +4830,7 @@
         <v>3</v>
       </c>
       <c r="M45" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>15</v>
       </c>
       <c r="N45" s="36">
@@ -4814,7 +4843,7 @@
         <v>0.001</v>
       </c>
       <c r="Q45" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.1</v>
       </c>
       <c r="R45" s="36"/>
@@ -4823,7 +4852,7 @@
     <row r="46" spans="1:19">
       <c r="A46" s="2"/>
       <c r="B46" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>37</v>
       </c>
       <c r="C46" s="38" t="s">
@@ -4844,7 +4873,9 @@
       <c r="H46" s="39" t="s">
         <v>39</v>
       </c>
-      <c r="I46" s="39"/>
+      <c r="I46" s="39" t="s">
+        <v>31</v>
+      </c>
       <c r="J46" s="39" t="s">
         <v>239</v>
       </c>
@@ -4855,7 +4886,7 @@
         <v>1</v>
       </c>
       <c r="M46" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N46" s="39">
@@ -4868,7 +4899,7 @@
         <v>0.0258</v>
       </c>
       <c r="Q46" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.516</v>
       </c>
       <c r="R46" s="39"/>
@@ -4877,7 +4908,7 @@
     <row r="47" spans="1:19">
       <c r="A47" s="2"/>
       <c r="B47" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>38</v>
       </c>
       <c r="C47" s="35" t="s">
@@ -4898,7 +4929,9 @@
       <c r="H47" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="I47" s="36"/>
+      <c r="I47" s="39" t="s">
+        <v>31</v>
+      </c>
       <c r="J47" s="36" t="s">
         <v>244</v>
       </c>
@@ -4909,7 +4942,7 @@
         <v>1</v>
       </c>
       <c r="M47" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N47" s="36">
@@ -4922,7 +4955,7 @@
         <v>0.0012</v>
       </c>
       <c r="Q47" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.12</v>
       </c>
       <c r="R47" s="36"/>
@@ -4931,7 +4964,7 @@
     <row r="48" spans="1:19">
       <c r="A48" s="2"/>
       <c r="B48" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>39</v>
       </c>
       <c r="C48" s="38" t="s">
@@ -4965,7 +4998,7 @@
         <v>6</v>
       </c>
       <c r="M48" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>30</v>
       </c>
       <c r="N48" s="39">
@@ -4978,7 +5011,7 @@
         <v>0.001</v>
       </c>
       <c r="Q48" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.1</v>
       </c>
       <c r="R48" s="39"/>
@@ -4987,7 +5020,7 @@
     <row r="49" ht="24" spans="1:19">
       <c r="A49" s="2"/>
       <c r="B49" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>40</v>
       </c>
       <c r="C49" s="35" t="s">
@@ -5008,7 +5041,9 @@
       <c r="H49" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="I49" s="36"/>
+      <c r="I49" s="36" t="s">
+        <v>31</v>
+      </c>
       <c r="J49" s="36" t="s">
         <v>258</v>
       </c>
@@ -5019,7 +5054,7 @@
         <v>2</v>
       </c>
       <c r="M49" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="N49" s="36">
@@ -5032,7 +5067,7 @@
         <v>0.1555</v>
       </c>
       <c r="Q49" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.3325</v>
       </c>
       <c r="R49" s="36"/>
@@ -5041,7 +5076,7 @@
     <row r="50" ht="24" spans="1:19">
       <c r="A50" s="2"/>
       <c r="B50" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>41</v>
       </c>
       <c r="C50" s="38" t="s">
@@ -5062,7 +5097,9 @@
       <c r="H50" s="39" t="s">
         <v>263</v>
       </c>
-      <c r="I50" s="39"/>
+      <c r="I50" s="36" t="s">
+        <v>31</v>
+      </c>
       <c r="J50" s="39" t="s">
         <v>264</v>
       </c>
@@ -5073,7 +5110,7 @@
         <v>1</v>
       </c>
       <c r="M50" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N50" s="39">
@@ -5086,7 +5123,7 @@
         <v>0.0927</v>
       </c>
       <c r="Q50" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>0.927</v>
       </c>
       <c r="R50" s="39"/>
@@ -5095,7 +5132,7 @@
     <row r="51" ht="24" spans="1:19">
       <c r="A51" s="2"/>
       <c r="B51" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>42</v>
       </c>
       <c r="C51" s="35" t="s">
@@ -5116,7 +5153,9 @@
       <c r="H51" s="36" t="s">
         <v>269</v>
       </c>
-      <c r="I51" s="36"/>
+      <c r="I51" s="36" t="s">
+        <v>31</v>
+      </c>
       <c r="J51" s="36" t="s">
         <v>270</v>
       </c>
@@ -5127,7 +5166,7 @@
         <v>2</v>
       </c>
       <c r="M51" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="N51" s="36">
@@ -5140,7 +5179,7 @@
         <v>0.3404</v>
       </c>
       <c r="Q51" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>4.0848</v>
       </c>
       <c r="R51" s="36"/>
@@ -5149,7 +5188,7 @@
     <row r="52" ht="24" spans="1:19">
       <c r="A52" s="2"/>
       <c r="B52" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>43</v>
       </c>
       <c r="C52" s="38" t="s">
@@ -5170,7 +5209,9 @@
       <c r="H52" s="39" t="s">
         <v>275</v>
       </c>
-      <c r="I52" s="39"/>
+      <c r="I52" s="39" t="s">
+        <v>31</v>
+      </c>
       <c r="J52" s="39" t="s">
         <v>276</v>
       </c>
@@ -5181,7 +5222,7 @@
         <v>2</v>
       </c>
       <c r="M52" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="N52" s="39">
@@ -5194,7 +5235,7 @@
         <v>0.0542</v>
       </c>
       <c r="Q52" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>1.084</v>
       </c>
       <c r="R52" s="39"/>
@@ -5203,7 +5244,7 @@
     <row r="53" ht="28.8" spans="1:19">
       <c r="A53" s="2"/>
       <c r="B53" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>44</v>
       </c>
       <c r="C53" s="35" t="s">
@@ -5237,7 +5278,7 @@
         <v>1</v>
       </c>
       <c r="M53" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N53" s="36">
@@ -5250,7 +5291,7 @@
         <v>2.76</v>
       </c>
       <c r="Q53" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>16.56</v>
       </c>
       <c r="R53" s="36"/>
@@ -5259,7 +5300,7 @@
     <row r="54" spans="1:19">
       <c r="A54" s="2"/>
       <c r="B54" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>45</v>
       </c>
       <c r="C54" s="38" t="s">
@@ -5280,7 +5321,9 @@
       <c r="H54" s="39" t="s">
         <v>288</v>
       </c>
-      <c r="I54" s="39"/>
+      <c r="I54" s="39" t="s">
+        <v>31</v>
+      </c>
       <c r="J54" s="39" t="s">
         <v>289</v>
       </c>
@@ -5291,7 +5334,7 @@
         <v>1</v>
       </c>
       <c r="M54" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N54" s="39">
@@ -5304,7 +5347,7 @@
         <v>0.114</v>
       </c>
       <c r="Q54" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>1.14</v>
       </c>
       <c r="R54" s="39"/>
@@ -5313,7 +5356,7 @@
     <row r="55" spans="1:19">
       <c r="A55" s="2"/>
       <c r="B55" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>46</v>
       </c>
       <c r="C55" s="35" t="s">
@@ -5347,7 +5390,7 @@
         <v>1</v>
       </c>
       <c r="M55" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N55" s="36">
@@ -5360,7 +5403,7 @@
         <v>0.1874</v>
       </c>
       <c r="Q55" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>1.874</v>
       </c>
       <c r="R55" s="36"/>
@@ -5369,7 +5412,7 @@
     <row r="56" ht="24" spans="1:19">
       <c r="A56" s="2"/>
       <c r="B56" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>47</v>
       </c>
       <c r="C56" s="38" t="s">
@@ -5396,12 +5439,14 @@
       <c r="J56" s="39" t="s">
         <v>300</v>
       </c>
-      <c r="K56" s="39"/>
+      <c r="K56" s="36" t="s">
+        <v>31</v>
+      </c>
       <c r="L56" s="39">
         <v>1</v>
       </c>
       <c r="M56" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N56" s="39">
@@ -5414,7 +5459,7 @@
         <v>2.3913</v>
       </c>
       <c r="Q56" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>14.3478</v>
       </c>
       <c r="R56" s="39"/>
@@ -5423,7 +5468,7 @@
     <row r="57" spans="1:19">
       <c r="A57" s="2"/>
       <c r="B57" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>48</v>
       </c>
       <c r="C57" s="35" t="s">
@@ -5442,34 +5487,36 @@
         <v>304</v>
       </c>
       <c r="H57" s="39" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="I57" s="36" t="s">
         <v>31</v>
       </c>
       <c r="J57" s="36" t="s">
-        <v>305</v>
-      </c>
-      <c r="K57" s="36"/>
+        <v>306</v>
+      </c>
+      <c r="K57" s="36" t="s">
+        <v>31</v>
+      </c>
       <c r="L57" s="36">
         <v>1</v>
       </c>
       <c r="M57" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N57" s="36">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O57" s="54" t="s">
         <v>34</v>
       </c>
       <c r="P57" s="55">
-        <v>0.8257</v>
+        <v>0.0755</v>
       </c>
       <c r="Q57" s="55">
-        <f t="shared" si="2"/>
-        <v>4.9542</v>
+        <f t="shared" si="5"/>
+        <v>0.755</v>
       </c>
       <c r="R57" s="36"/>
       <c r="S57" s="65"/>
@@ -5477,39 +5524,41 @@
     <row r="58" ht="24" spans="1:19">
       <c r="A58" s="2"/>
       <c r="B58" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>49</v>
       </c>
       <c r="C58" s="38" t="s">
         <v>294</v>
       </c>
       <c r="D58" s="39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="E58" s="39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="F58" s="39" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="G58" s="39" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H58" s="39" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="I58" s="36" t="s">
         <v>31</v>
       </c>
       <c r="J58" s="39" t="s">
-        <v>311</v>
-      </c>
-      <c r="K58" s="39"/>
+        <v>312</v>
+      </c>
+      <c r="K58" s="36" t="s">
+        <v>31</v>
+      </c>
       <c r="L58" s="39">
         <v>1</v>
       </c>
       <c r="M58" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N58" s="39">
@@ -5522,32 +5571,32 @@
         <v>1.1384</v>
       </c>
       <c r="Q58" s="57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>6.8304</v>
       </c>
       <c r="R58" s="39"/>
       <c r="S58" s="39"/>
     </row>
-    <row r="59" ht="15.15" spans="1:19">
+    <row r="59" spans="1:19">
       <c r="A59" s="2"/>
       <c r="B59" s="34">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>50</v>
       </c>
       <c r="C59" s="35" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D59" s="36" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E59" s="36" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F59" s="36" t="s">
         <v>168</v>
       </c>
       <c r="G59" s="36" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="H59" s="36" t="s">
         <v>170</v>
@@ -5556,14 +5605,16 @@
         <v>31</v>
       </c>
       <c r="J59" s="36" t="s">
-        <v>316</v>
-      </c>
-      <c r="K59" s="36"/>
+        <v>317</v>
+      </c>
+      <c r="K59" s="36" t="s">
+        <v>31</v>
+      </c>
       <c r="L59" s="36">
         <v>1</v>
       </c>
       <c r="M59" s="36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="N59" s="36">
@@ -5576,7 +5627,7 @@
         <v>0.2156</v>
       </c>
       <c r="Q59" s="55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="5"/>
         <v>2.156</v>
       </c>
       <c r="R59" s="36"/>
@@ -5597,13 +5648,13 @@
       <c r="L60" s="48"/>
       <c r="M60" s="48"/>
       <c r="N60" s="59" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="O60" s="60"/>
       <c r="P60" s="60"/>
       <c r="Q60" s="67">
         <f>SUM(Q10:Q59)</f>
-        <v>116.1864</v>
+        <v>111.9872</v>
       </c>
       <c r="R60" s="68"/>
       <c r="S60" s="69"/>
@@ -5623,13 +5674,13 @@
       <c r="L61" s="52"/>
       <c r="M61" s="52"/>
       <c r="N61" s="59" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="O61" s="60"/>
       <c r="P61" s="60"/>
       <c r="Q61" s="70">
         <f>Q60/5</f>
-        <v>23.23728</v>
+        <v>22.39744</v>
       </c>
       <c r="R61" s="71"/>
       <c r="S61" s="72"/>
@@ -5689,8 +5740,8 @@
     <hyperlink ref="O48" r:id="rId44" display="LCSC"/>
     <hyperlink ref="O53" r:id="rId45" display="Aliexpress"/>
     <hyperlink ref="O55" r:id="rId46" display="LCSC"/>
-    <hyperlink ref="O57" r:id="rId47" display="LCSC"/>
-    <hyperlink ref="O19" r:id="rId48" display="LCSC"/>
+    <hyperlink ref="O19" r:id="rId47" display="LCSC"/>
+    <hyperlink ref="O57" r:id="rId48" display="LCSC"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>